<commit_message>
Replaced Joseph dataset after correcting material in fiber material in the .xlsx
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Bernaert_2024-09_QS/TST_2024-09_QS_metadata.xlsx
+++ b/Data/raw/TST_Bernaert_2024-09_QS/TST_2024-09_QS_metadata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Bernaert_2024-09_QS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4381A189-6737-42FB-BC0C-005BF03C260A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D649E933-C538-4023-8741-E885D342B13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiment" sheetId="1" r:id="rId1"/>
@@ -266,9 +266,6 @@
     <t>Hardener</t>
   </si>
   <si>
-    <t>Material</t>
-  </si>
-  <si>
     <t>Sequential number</t>
   </si>
   <si>
@@ -345,6 +342,9 @@
   </si>
   <si>
     <t>Polyester</t>
+  </si>
+  <si>
+    <t>Fiber Material</t>
   </si>
 </sst>
 </file>
@@ -1161,7 +1161,7 @@
         <v>1</v>
       </c>
       <c r="Q1" s="19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R1" s="19"/>
       <c r="S1" s="19"/>
@@ -1249,7 +1249,7 @@
         <v>57</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="U2" s="4" t="s">
         <v>58</v>
@@ -1311,13 +1311,13 @@
     </row>
     <row r="3" spans="1:39" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>94</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>20</v>
@@ -1341,7 +1341,7 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P3" s="5">
         <v>123</v>
@@ -1350,23 +1350,23 @@
         <v>47</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="S3" s="7"/>
       <c r="T3" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="U3" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>102</v>
       </c>
       <c r="V3" s="6"/>
       <c r="W3" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="X3" s="6"/>
       <c r="Y3" s="6"/>
       <c r="Z3" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
@@ -1526,43 +1526,43 @@
     </row>
     <row r="2" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -1570,7 +1570,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -1599,7 +1599,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -1628,7 +1628,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>

</xml_diff>

<commit_message>
Added L' and t to the database and changed all the files linked to the database. Added L' and t to the tests sheet in the metadata file. Changed also the calculation to account for both piano hinge and endblock
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Bernaert_2024-09_QS/TST_2024-09_QS_metadata.xlsx
+++ b/Data/raw/TST_Bernaert_2024-09_QS/TST_2024-09_QS_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Bernaert_2024-09_QS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D649E933-C538-4023-8741-E885D342B13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D29946C-7170-4B67-BD8A-8E4FAC6F3DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="15" windowWidth="20640" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiment" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="106">
   <si>
     <t>General</t>
   </si>
@@ -345,6 +345,12 @@
   </si>
   <si>
     <t>Fiber Material</t>
+  </si>
+  <si>
+    <t>L'</t>
+  </si>
+  <si>
+    <t>t</t>
   </si>
 </sst>
 </file>
@@ -493,7 +499,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -531,6 +537,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -556,7 +565,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -698,23 +714,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>308162</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>1232648</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>44823</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>1621744</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>76487</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>210865</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>976</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC0C11FC-D7EF-49B6-9CF8-E8BD18A71247}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1B9508C-222C-4C33-8061-B0765BCA93A4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -730,8 +746,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="23429633" y="3585883"/>
-          <a:ext cx="6096851" cy="3391373"/>
+          <a:off x="26587824" y="1822823"/>
+          <a:ext cx="5679186" cy="2167410"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1140,55 +1156,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
       <c r="P1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="Q1" s="19" t="s">
+      <c r="Q1" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-      <c r="T1" s="19"/>
-      <c r="U1" s="19"/>
-      <c r="V1" s="19"/>
-      <c r="W1" s="19"/>
-      <c r="X1" s="19"/>
-      <c r="Y1" s="19"/>
-      <c r="Z1" s="19"/>
-      <c r="AA1" s="19"/>
-      <c r="AB1" s="19"/>
-      <c r="AC1" s="19"/>
-      <c r="AD1" s="19"/>
-      <c r="AE1" s="19"/>
-      <c r="AF1" s="19"/>
-      <c r="AG1" s="19"/>
-      <c r="AH1" s="19"/>
-      <c r="AI1" s="19"/>
-      <c r="AJ1" s="17" t="s">
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="20"/>
+      <c r="Z1" s="20"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="20"/>
+      <c r="AC1" s="20"/>
+      <c r="AD1" s="20"/>
+      <c r="AE1" s="20"/>
+      <c r="AF1" s="20"/>
+      <c r="AG1" s="20"/>
+      <c r="AH1" s="20"/>
+      <c r="AI1" s="20"/>
+      <c r="AJ1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="AK1" s="17"/>
-      <c r="AL1" s="15" t="s">
+      <c r="AK1" s="18"/>
+      <c r="AL1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="AM1" s="16"/>
+      <c r="AM1" s="17"/>
     </row>
     <row r="2" spans="1:39" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
@@ -1395,32 +1411,32 @@
     <mergeCell ref="Q1:AI1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>D3="QS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3 M3 AL3:AM3">
-    <cfRule type="expression" dxfId="6" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>$D$3="FA"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>D3="OT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3 N3">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>G3="Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>OR(E3="fracture", F3="fracture")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S3">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>Q3="Other polymers"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1481,7 +1497,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.33203125" style="3" customWidth="1"/>
@@ -1491,40 +1507,42 @@
     <col min="5" max="5" width="39.88671875" style="3" customWidth="1"/>
     <col min="6" max="6" width="19.109375" style="3" customWidth="1"/>
     <col min="7" max="7" width="19.88671875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="20.5546875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="20.109375" style="3" customWidth="1"/>
-    <col min="10" max="11" width="15.6640625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="21.88671875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="20" style="3" customWidth="1"/>
-    <col min="14" max="16384" width="8.6640625" style="3"/>
+    <col min="8" max="10" width="20.5546875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="20.109375" style="3" customWidth="1"/>
+    <col min="12" max="13" width="15.6640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="21.88671875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="20" style="3" customWidth="1"/>
+    <col min="16" max="16384" width="8.6640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="21" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="19" t="s">
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="17" t="s">
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="K1" s="17"/>
-      <c r="L1" s="20" t="s">
+      <c r="M1" s="18"/>
+      <c r="N1" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="M1" s="20"/>
-    </row>
-    <row r="2" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O1" s="21"/>
+    </row>
+    <row r="2" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>77</v>
       </c>
@@ -1553,19 +1571,25 @@
         <v>85</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -1585,16 +1609,22 @@
       <c r="I3" s="6">
         <v>50</v>
       </c>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="6">
+      <c r="J3" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" s="6">
+        <v>22</v>
+      </c>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="6">
         <v>35</v>
       </c>
-      <c r="M3" s="6">
+      <c r="O3" s="6">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>2</v>
       </c>
@@ -1614,16 +1644,22 @@
       <c r="I4" s="13">
         <v>51</v>
       </c>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="13">
+      <c r="J4" s="15">
+        <v>0</v>
+      </c>
+      <c r="K4" s="13">
+        <v>22</v>
+      </c>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="13">
         <v>35</v>
       </c>
-      <c r="M4" s="13">
+      <c r="O4" s="13">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>3</v>
       </c>
@@ -1643,76 +1679,82 @@
       <c r="I5" s="13">
         <v>50.5</v>
       </c>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="13">
+      <c r="J5" s="15">
+        <v>0</v>
+      </c>
+      <c r="K5" s="13">
+        <v>22</v>
+      </c>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="13">
         <v>35</v>
       </c>
-      <c r="M5" s="13">
+      <c r="O5" s="13">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="D16" s="1"/>
@@ -1763,11 +1805,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="5">
-    <mergeCell ref="J1:K1"/>
     <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:O1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F1:K1"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75" bottom="0.75" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -1776,7 +1818,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="2" id="{16E6D065-EB34-40AF-805E-2A054E24FEF5}">
+          <x14:cfRule type="expression" priority="3" id="{16E6D065-EB34-40AF-805E-2A054E24FEF5}">
             <xm:f>Experiment!$D$3="FA"</xm:f>
             <x14:dxf>
               <fill>
@@ -1789,7 +1831,7 @@
           <xm:sqref>C3:E5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="1" id="{3B68649E-35DF-4270-8AEE-1821476DDEC7}">
+          <x14:cfRule type="expression" priority="1" id="{8C74D885-4D99-4FE5-A519-3E7045908205}">
             <xm:f>OR(Experiment!E$3="fracture", Experiment!F$3="fracture")</xm:f>
             <x14:dxf>
               <fill>
@@ -1800,6 +1842,19 @@
             </x14:dxf>
           </x14:cfRule>
           <xm:sqref>I3:I5</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="2" id="{3B68649E-35DF-4270-8AEE-1821476DDEC7}">
+            <xm:f>OR(Experiment!G$3="fracture", Experiment!H$3="fracture")</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>K3:K5</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Checked the code for fracture energies with Joseph and corrected the t values in the excel file
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Bernaert_2024-09_QS/TST_2024-09_QS_metadata.xlsx
+++ b/Data/raw/TST_Bernaert_2024-09_QS/TST_2024-09_QS_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Bernaert_2024-09_QS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D29946C-7170-4B67-BD8A-8E4FAC6F3DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CFC57E7-14D7-4DFC-ACF3-EF1E61B07FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15" windowWidth="20640" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1613,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="6">
-        <v>22</v>
+        <v>27.53</v>
       </c>
       <c r="L3" s="11"/>
       <c r="M3" s="11"/>
@@ -1648,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="13">
-        <v>22</v>
+        <v>27.440999999999999</v>
       </c>
       <c r="L4" s="14"/>
       <c r="M4" s="14"/>
@@ -1683,7 +1683,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="13">
-        <v>22</v>
+        <v>27.57</v>
       </c>
       <c r="L5" s="14"/>
       <c r="M5" s="14"/>

</xml_diff>